<commit_message>
feat: complete role B D27 deliverables
</commit_message>
<xml_diff>
--- a/progress_时间节点已修正.xlsx
+++ b/progress_时间节点已修正.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progress" sheetId="1" r:id="Rad8b30b886ae4893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progress" sheetId="1" r:id="Re0c18ed5ad3446d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -930,7 +930,7 @@
         <x:color rgb="FF2E6B2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -941,7 +941,7 @@
         <x:color rgb="FF1F4E78"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBF7"/>
         </x:patternFill>
       </x:fill>
@@ -952,7 +952,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -963,7 +963,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -973,7 +973,7 @@
         <x:color rgb="FF666666"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -984,7 +984,7 @@
         <x:color rgb="FF2E6B2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -995,7 +995,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1005,7 +1005,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1414,7 +1414,7 @@
         <x:v>D27-01</x:v>
       </x:c>
       <x:c r="H4" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I4" s="35" t="str">
         <x:v>data/raw/A题数据集.csv；data/legacy/；docs/data_inventory.csv</x:v>
@@ -1423,19 +1423,19 @@
         <x:v>官方原始数据只有一个只读版本；三份历史清洗均能追溯到人员和代码</x:v>
       </x:c>
       <x:c r="K4" s="35" t="str">
-        <x:v>待填写：原始数据行列数及三份清洗差异</x:v>
+        <x:v>原始数据10,000×64，数据清单已生成；未发现三份可追溯历史清洗</x:v>
       </x:c>
       <x:c r="L4" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>缺data/legacy三份历史清洗及人员/代码追溯</x:v>
       </x:c>
       <x:c r="M4" s="33" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N4" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O4" s="35" t="str">
-        <x:v>完成数据清单后立即支持公共清洗复核</x:v>
+        <x:v>A补齐data/legacy三份历史结果后由B复核</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1461,7 +1461,7 @@
         <x:v>D27-02</x:v>
       </x:c>
       <x:c r="H5" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I5" s="35" t="str">
         <x:v>docs/cleaning_comparison.csv；config/cleaning_spec.yaml</x:v>
@@ -1470,19 +1470,19 @@
         <x:v>Alcohol缺失→Unknown；运动相关语义缺失按规则修复；公共表不编码、不标准化、不截断、不删行；禁止手改CSV</x:v>
       </x:c>
       <x:c r="K5" s="35" t="str">
-        <x:v>待填写：三人确认的最终规则</x:v>
+        <x:v>规则已锁定：Unknown、No Exercise、No Workout；公共表固定66列</x:v>
       </x:c>
       <x:c r="L5" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>缺docs/cleaning_comparison.csv及三版来源证据</x:v>
       </x:c>
       <x:c r="M5" s="33" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N5" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O5" s="35" t="str">
-        <x:v>规则PASS后由A生成公共清洗数据</x:v>
+        <x:v>A补齐三版对比后由三人确认</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1508,7 +1508,7 @@
         <x:v>D27-01</x:v>
       </x:c>
       <x:c r="H6" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>待复核</x:v>
       </x:c>
       <x:c r="I6" s="35" t="str">
         <x:v>config/targets.yaml；config/leakage_blacklist.yaml；docs/metrics_schema.csv</x:v>
@@ -1517,19 +1517,19 @@
         <x:v>三任务X/y明确；任务二四档边界明确；各任务泄漏字段及理由明确；评价指标口径统一</x:v>
       </x:c>
       <x:c r="K6" s="35" t="str">
-        <x:v>待填写：三任务标签与泄漏字段</x:v>
+        <x:v>三任务标签、固定类别顺序、Task2四档边界、统一指标字段及泄漏原因已配置</x:v>
       </x:c>
       <x:c r="L6" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>B交付完成；Task2边界口径D-016待三人复核</x:v>
       </x:c>
       <x:c r="M6" s="33" t="str">
         <x:v>待复核</x:v>
       </x:c>
       <x:c r="N6" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O6" s="35" t="str">
-        <x:v>配置PASS后完成统一标签和评价函数</x:v>
+        <x:v>三人复核targets/leakage/metrics schema</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1555,28 +1555,28 @@
         <x:v>D27-03</x:v>
       </x:c>
       <x:c r="H7" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="I7" s="35" t="str">
         <x:v>src/preprocess.py；data/processed/base_semantic_clean.csv；results/data_audit/cleaning_validation.csv</x:v>
       </x:c>
       <x:c r="J7" s="35" t="str">
-        <x:v>10,000行×64列；保留Person_ID；Alcohol原缺失均为Unknown；原始非缺失值未改；验证项全部PASS</x:v>
+        <x:v>10,000行×66列（64个原始字段＋2个分钟衍生字段）；保留Person_ID；Alcohol原缺失均为Unknown；原始非缺失值未改；验证项全部PASS</x:v>
       </x:c>
       <x:c r="K7" s="35" t="str">
-        <x:v>待填写：行列数、Unknown数量及验证结论</x:v>
+        <x:v>10,000×66；0缺失；Person_ID唯一；Unknown=3014；No Exercise=824；No Workout=824；20/20验证PASS；全套45项测试通过</x:v>
       </x:c>
       <x:c r="L7" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>已解决：D-015统一64原始列＋2分钟衍生列</x:v>
       </x:c>
       <x:c r="M7" s="33" t="str">
-        <x:v>待复核</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N7" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O7" s="35" t="str">
-        <x:v>公共清洗、标签、泄漏和切分全部PASS后，三任务同时启动</x:v>
+        <x:v>公共清洗PASS；继续统一标签与三任务基线</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1602,7 +1602,7 @@
         <x:v>D27-04</x:v>
       </x:c>
       <x:c r="H8" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>待复核</x:v>
       </x:c>
       <x:c r="I8" s="35" t="str">
         <x:v>src/targets.py；src/evaluate.py；tests/test_targets_evaluate.py</x:v>
@@ -1611,19 +1611,19 @@
         <x:v>标签类别、顺序和分档边界正确；Accuracy、Macro-F1、Balanced Accuracy及任务附加指标可统一输出</x:v>
       </x:c>
       <x:c r="K8" s="35" t="str">
-        <x:v>待填写：单元测试结果</x:v>
+        <x:v>统一标签/编码/解码、泄漏检查和各任务指标已实现；新增10项测试，全套45/45通过</x:v>
       </x:c>
       <x:c r="L8" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>B交付完成，待C复核</x:v>
       </x:c>
       <x:c r="M8" s="33" t="str">
         <x:v>待复核</x:v>
       </x:c>
       <x:c r="N8" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O8" s="35" t="str">
-        <x:v>三任务统一调用，不得各自另写指标口径</x:v>
+        <x:v>C复核后作为三任务唯一评价接口</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1649,7 +1649,7 @@
         <x:v>D27-04；D27-05</x:v>
       </x:c>
       <x:c r="H9" s="33" t="str">
-        <x:v>未开始</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="I9" s="35" t="str">
         <x:v>src/split.py；data/splits/split_manifest.csv；tests/test_split.py</x:v>
@@ -1658,19 +1658,19 @@
         <x:v>seed=20260726；Person_ID唯一连接；三任务共用同一split；各类别分布合理；后续不得私自重切</x:v>
       </x:c>
       <x:c r="K9" s="35" t="str">
-        <x:v>待填写：训练/验证/测试行数及类别分布</x:v>
+        <x:v>seed=20260726；train=8,000，val=2,000；Person_ID 10,000唯一；9项切分测试PASS</x:v>
       </x:c>
       <x:c r="L9" s="35" t="str">
-        <x:v>待填写</x:v>
+        <x:v>无；Task2验证集ID完全一致且与训练集交集为0</x:v>
       </x:c>
       <x:c r="M9" s="33" t="str">
-        <x:v>待复核</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N9" s="36" t="n">
-        <x:v>46230.791666666664</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O9" s="35" t="str">
-        <x:v>切分PASS后，18:30—21:00运行三任务基线</x:v>
+        <x:v>三任务必须使用该split_manifest.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1696,7 +1696,7 @@
         <x:v>D27-05；D27-06；D27-07</x:v>
       </x:c>
       <x:c r="H10" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
         <x:v>src/task1.py；results/metrics/raw/task1_baseline.csv；results/figures/baseline/task1_confusion_matrix.png</x:v>
@@ -1705,19 +1705,19 @@
         <x:v>至少含Dummy和Logistic；报告Accuracy、Macro-F1、Balanced Accuracy、ROC-AUC和混淆矩阵；主结果不含泄漏字段</x:v>
       </x:c>
       <x:c r="K10" s="14" t="str">
-        <x:v>待填写：ACC1、Macro-F1、ROC-AUC</x:v>
+        <x:v>未收到task1_baseline.csv与任务一混淆矩阵</x:v>
       </x:c>
       <x:c r="L10" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>正式验收产物缺失，B无法复核</x:v>
       </x:c>
       <x:c r="M10" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N10" s="23" t="n">
-        <x:v>46230.9375</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O10" s="14" t="str">
-        <x:v>7月28日比较主模型并完成泄漏消融</x:v>
+        <x:v>A按统一接口和公共split补齐后交B复核</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1743,7 +1743,7 @@
         <x:v>D27-05；D27-06；D27-07</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>待复核</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
         <x:v>src/task2.py；results/metrics/raw/task2_baseline.csv；results/figures/baseline/task2_confusion_matrix.png</x:v>
@@ -1752,19 +1752,19 @@
         <x:v>至少含Dummy和线性/逻辑基线；报告Accuracy、Macro-F1、Balanced Accuracy、MAE、RMSE和混淆矩阵</x:v>
       </x:c>
       <x:c r="K11" s="14" t="str">
-        <x:v>待填写：ACC2、Macro-F1、MAE、RMSE</x:v>
+        <x:v>LR：ACC2=0.8265；Macro-F1=0.8202；BalAcc=0.8123；MAE=0.1735；RMSE=0.4165；Dummy ACC=0.4455</x:v>
       </x:c>
       <x:c r="L11" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>B交付完成，公共2,000验证集已独立对账，待C复核</x:v>
       </x:c>
       <x:c r="M11" s="17" t="str">
         <x:v>待复核</x:v>
       </x:c>
       <x:c r="N11" s="23" t="n">
-        <x:v>46230.9375</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O11" s="14" t="str">
-        <x:v>7月28日比较回归后分档与直接分类</x:v>
+        <x:v>C复核指标CSV和混淆矩阵；7/28比较回归后分档</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1837,28 +1837,28 @@
         <x:v>D27-08；D27-09；D27-10</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>results/metrics/baseline_raw.csv；results/issues/issues_0727.md；decision_log.md</x:v>
+        <x:v>results/metrics/baseline_raw.csv；results/issues/issues_0727.md；docs/decision_log.md</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
         <x:v>三个任务的指标字段、类别顺序、样本量和seed一致；问题写清负责人和最晚修复时间</x:v>
       </x:c>
       <x:c r="K13" s="14" t="str">
-        <x:v>待填写：ACC1/ACC2/ACC3及三项Macro-F1</x:v>
+        <x:v>Task2正式基线已完成；Task1/Task3指标未收到，未生成不完整baseline_raw.csv</x:v>
       </x:c>
       <x:c r="L13" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>I-0727-01/02：缺A/C基线；详见results/issues/issues_0727.md</x:v>
       </x:c>
       <x:c r="M13" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N13" s="23" t="n">
-        <x:v>46230.9583333333</x:v>
+        <x:v>46230.94957175926</x:v>
       </x:c>
       <x:c r="O13" s="14" t="str">
-        <x:v>若基线FAIL，先修基线，不启动额外调参</x:v>
+        <x:v>A/C补齐正式基线后由B合并并重新验收</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -3435,7 +3435,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re56fb8a878264909"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5440c3f0d6ea4544"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete role B D28 model comparison
</commit_message>
<xml_diff>
--- a/progress_时间节点已修正.xlsx
+++ b/progress_时间节点已修正.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progress" sheetId="1" r:id="Re0c18ed5ad3446d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="progress" sheetId="1" r:id="R2c3e7a339ea54fcc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1884,7 +1884,7 @@
         <x:v>D27-08；D27-11</x:v>
       </x:c>
       <x:c r="H14" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
         <x:v>results/metrics/raw/task1_model_comparison.csv；results/metrics/raw/task1_leakage_ablation.csv</x:v>
@@ -1893,19 +1893,19 @@
         <x:v>同一split和seed；比较基线、主模型和一个对比模型；分别展示含直接泄漏、删除直接泄漏、删除可重构字段的结果</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
-        <x:v>待填写：最佳无泄漏模型及消融差异</x:v>
+        <x:v>未收到Task1模型比较与泄漏消融正式CSV</x:v>
       </x:c>
       <x:c r="L14" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>A产物未到，B无法执行泄漏消融复核</x:v>
       </x:c>
       <x:c r="M14" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N14" s="23" t="n">
-        <x:v>46231.75</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O14" s="14" t="str">
-        <x:v>提交最终模型候选和推荐理由</x:v>
+        <x:v>A补齐三组泄漏消融后交B复核</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1931,28 +1931,28 @@
         <x:v>D27-09；D27-11</x:v>
       </x:c>
       <x:c r="H15" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>results/metrics/raw/task2_model_comparison.csv；results/metrics/raw/task2_method_ablation.csv</x:v>
+        <x:v>results/metrics/raw/task2_model_comparison.csv；results/metrics/raw/task2_method_ablation.csv；results/metrics/raw/task2_tuning_log.csv</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str">
         <x:v>同一split和seed；比较回归后分档与直接分类；同时报告分类指标和MAE/RMSE</x:v>
       </x:c>
       <x:c r="K15" s="14" t="str">
-        <x:v>待填写：两种路线优劣及候选模型</x:v>
+        <x:v>六模型族/16配置；Ridge回归分档：ACC=0.8340，Macro-F1=0.8244，BalAcc=0.8145，MAE=0.1660，RMSE=0.4074；优于直接LR ACC=0.8265</x:v>
       </x:c>
       <x:c r="L15" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>B交付完成；指标独立重算一致，待C复核</x:v>
       </x:c>
       <x:c r="M15" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="N15" s="23" t="n">
-        <x:v>46231.75</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O15" s="14" t="str">
-        <x:v>提交最终模型候选和推荐理由</x:v>
+        <x:v>C复核两条路线、CSV与2,000行预测；冻结前再确认</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2025,7 +2025,7 @@
         <x:v>D28-01；D28-02；D28-03</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I17" s="14" t="str">
         <x:v>results/metrics/model_comparison.csv；results/metrics/tuning_log.csv；results/metrics/ablation.csv</x:v>
@@ -2034,19 +2034,19 @@
         <x:v>每行包含task、数据版本、split、seed、模型、参数、指标、运行时间和输出路径；无重复口径</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
-        <x:v>待填写：三个任务的候选排名</x:v>
+        <x:v>Task2比较/调参/消融已齐；严格聚合门禁按预期拒绝生成不完整全任务CSV</x:v>
       </x:c>
       <x:c r="L17" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>缺Task1/Task3模型比较及消融正式CSV</x:v>
       </x:c>
       <x:c r="M17" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N17" s="23" t="n">
-        <x:v>46231.7708333333</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O17" s="14" t="str">
-        <x:v>20:30前形成最终配置建议</x:v>
+        <x:v>A/C补齐后由B运行三任务聚合并形成最终配置建议</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2072,7 +2072,7 @@
         <x:v>D28-04</x:v>
       </x:c>
       <x:c r="H18" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I18" s="14" t="str">
         <x:v>results/logs/reproduction_candidates.md；results/logs/candidate_runs/</x:v>
@@ -2081,19 +2081,19 @@
         <x:v>另一环境可运行；数据、split、seed和配置一致；指标允许小数误差但结论不变</x:v>
       </x:c>
       <x:c r="K18" s="14" t="str">
-        <x:v>待填写：复现PASS/FAIL及差异</x:v>
+        <x:v>未收到三任务入围候选复现报告</x:v>
       </x:c>
       <x:c r="L18" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>D28-04未完成，无法按1e-4容差复核</x:v>
       </x:c>
       <x:c r="M18" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N18" s="23" t="n">
-        <x:v>46231.8125</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O18" s="14" t="str">
-        <x:v>FAIL项先修复，再参加冻结评审</x:v>
+        <x:v>A完成复现后交B核对数据、split、seed和指标</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="14" hidden="0" customHeight="1">
@@ -2119,7 +2119,7 @@
         <x:v>D28-01；D28-02；D28-03</x:v>
       </x:c>
       <x:c r="H19" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I19" s="14" t="str">
         <x:v>results/figures/candidate/；paper/figures/captions_draft.md</x:v>
@@ -2128,19 +2128,19 @@
         <x:v>图名、类别顺序、坐标和模型版本正确；每张图能追溯到输入和生成脚本</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
-        <x:v>待填写：候选图清单</x:v>
+        <x:v>未收到候选图、特征重要性与图注</x:v>
       </x:c>
       <x:c r="L19" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>缺C正式产物，B无法追溯输入/脚本/模型版本</x:v>
       </x:c>
       <x:c r="M19" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N19" s="23" t="n">
-        <x:v>46231.8125</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O19" s="14" t="str">
-        <x:v>冻结时确定最终图表清单</x:v>
+        <x:v>C补齐后由B复核类别顺序、轴标签和可追溯性</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2166,7 +2166,7 @@
         <x:v>D28-04；D28-05</x:v>
       </x:c>
       <x:c r="H20" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>待复核</x:v>
       </x:c>
       <x:c r="I20" s="14" t="str">
         <x:v>config/final/task1.yaml；config/final/task2.yaml；config/final/task3.yaml；docs/final_model_decision.md</x:v>
@@ -2175,19 +2175,19 @@
         <x:v>每个配置写明数据、标签、特征、模型、参数、类别权重和seed；选择理由兼顾无泄漏、主指标、少数类、稳定性和解释性</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
-        <x:v>待填写：三个最终模型及核心参数</x:v>
+        <x:v>Task2当前候选为Ridge回归后分档；三任务最终配置尚未齐备</x:v>
       </x:c>
       <x:c r="L20" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>依赖D28-04/D28-05及三人确认</x:v>
       </x:c>
       <x:c r="M20" s="17" t="str">
         <x:v>待复核</x:v>
       </x:c>
       <x:c r="N20" s="23" t="n">
-        <x:v>46231.9166666667</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O20" s="14" t="str">
-        <x:v>三人签字后禁止换模型或新增特征</x:v>
+        <x:v>三任务聚合与复现PASS后由三人评审最终配置</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="14" hidden="0" customHeight="1">
@@ -2213,7 +2213,7 @@
         <x:v>D28-07</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>待复核</x:v>
       </x:c>
       <x:c r="I21" s="14" t="str">
         <x:v>config/final/freeze_manifest.yaml；decision_log.md</x:v>
@@ -2222,19 +2222,19 @@
         <x:v>数据版本、标签、泄漏字段、split、模型、参数、权重、seed和代码版本全部锁定</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
-        <x:v>待填写：冻结版本号与三人确认</x:v>
+        <x:v>冻结门禁未满足，未生成freeze_manifest.yaml</x:v>
       </x:c>
       <x:c r="L21" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>缺三任务最终配置、复现PASS和三人签字</x:v>
       </x:c>
       <x:c r="M21" s="17" t="str">
         <x:v>待复核</x:v>
       </x:c>
       <x:c r="N21" s="23" t="n">
-        <x:v>46231.9166666667</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O21" s="14" t="str">
-        <x:v>冻结后仅修明确错误，不再试参</x:v>
+        <x:v>D28-07三人确认后再记录数据/配置/代码哈希</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2260,7 +2260,7 @@
         <x:v>D28-06；D28-07</x:v>
       </x:c>
       <x:c r="H22" s="17" t="str">
-        <x:v>未开始</x:v>
+        <x:v>阻塞</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
         <x:v>results/final/figure_manifest.csv</x:v>
@@ -2269,19 +2269,19 @@
         <x:v>每张正式图写明task、模型、输入、生成脚本、文件名和论文位置；不再增加展示模型</x:v>
       </x:c>
       <x:c r="K22" s="14" t="str">
-        <x:v>待填写：最终图表数量</x:v>
+        <x:v>未收到results/final/figure_manifest.csv</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
-        <x:v>待填写</x:v>
+        <x:v>D28-06/D28-07未完成，B无法复核最终图表清单</x:v>
       </x:c>
       <x:c r="M22" s="17" t="str">
-        <x:v>待复核</x:v>
+        <x:v>FAIL</x:v>
       </x:c>
       <x:c r="N22" s="23" t="n">
-        <x:v>46231.9166666667</x:v>
+        <x:v>46231.729166666664</x:v>
       </x:c>
       <x:c r="O22" s="14" t="str">
-        <x:v>只从冻结后的正式结果生成图表</x:v>
+        <x:v>C提交图表清单后由B复核输入、脚本和论文位置</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -3435,7 +3435,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5440c3f0d6ea4544"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4f0936a3ac4493a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>